<commit_message>
Reglas con envoltorios heredados: desmontaje compartido para Generate, import y migración
El desmontaje que solo aplicaba Generate pasa a una función compartida
(rule_wrappers.py y su gemela ruleWrappers.js, con los mismos casos): la
usan los tres generadores, el import de Excel (guarda la regla ya limpia) y
normalize_rule_wrappers.py (limpia lo guardado, con --dry-run y entrada en el
historial). La plantilla 4.2 queda limpia (S1-00070, S1-00507). El test no
se hace más tolerante.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rwcp9cSck72V1zULNhL8wU
</commit_message>
<xml_diff>
--- a/public/brdp-template-4-2.xlsx
+++ b/public/brdp-template-4-2.xlsx
@@ -622,16 +622,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>&lt;rules&gt;
-&lt;structureObjectRule&gt;
+          <t>&lt;structureObjectRule&gt;
             &lt;objectPath allowedObjectFlag="0"&gt;//randomList//randomList&lt;/objectPath&gt;
             &lt;objectUse&gt;BRDP-S1-00507. A &amp;lt;randomList&amp;gt; must not be nested inside another &amp;lt;randomList&amp;gt; -- the default prefix pf02 is always used, without nesting. &lt;/objectUse&gt;
           &lt;/structureObjectRule&gt;
 &lt;nonContextRule&gt;
           &lt;simplePara&gt;BRDP-S1-00507. Decide whether to use a consistent set of prefixes for random list throughout the project. &lt;/simplePara&gt;
           &lt;simplePara&gt;Decision made by Project. Nested randomList should be avoided. The listItemPrefix attribute shall always be the default value, which is pf02.&lt;/simplePara&gt;
-        &lt;/nonContextRule&gt;
-&lt;/rules&gt;</t>
+        &lt;/nonContextRule&gt;</t>
         </is>
       </c>
     </row>
@@ -708,8 +706,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>&lt;structureObjectRuleGroup&gt;
-&lt;structureObjectRule&gt;
+          <t>&lt;structureObjectRule&gt;
             &lt;objectPath allowedObjectFlag="1"&gt;//responsiblePartnerCompany/@enterpriseCode&lt;/objectPath&gt;
             &lt;objectUse&gt;BRDP-S1-00070. The responsible partner company's enterpriseCode must be C1008 (Lufthansa Technik AG's CAGE code). &lt;/objectUse&gt;
             &lt;objectValue valueForm="single" valueAllowed="C1008"&gt;CAGE code for LUFTHANSA TECHNIK AG is C1008&lt;/objectValue&gt;
@@ -718,8 +715,7 @@
             &lt;objectPath allowedObjectFlag="1"&gt;//responsiblePartnerCompany/enterpriseName&lt;/objectPath&gt;
             &lt;objectUse&gt;BRDP-S1-00070. The responsible partner company's enterpriseName must be 'LUFTHANSA TECHNIK AG'. &lt;/objectUse&gt;
             &lt;objectValue valueForm="single" valueAllowed="LUFTHANSA TECHNIK AG"&gt;Enterprise Name is LUFTHANSA TECHNIK AG&lt;/objectValue&gt;
-          &lt;/structureObjectRule&gt;
-&lt;/structureObjectRuleGroup&gt;</t>
+          &lt;/structureObjectRule&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Test de reglas: camino válido para anidar, S1-00338 por caracteres y aviso de ejemplos editados
- A//B en la ruta de la regla: el prompt da el anidamiento válido más corto
  según el grafo del esquema (randomList/listItem/para/randomList) y la
  ronda de corrección lo repite, con "keep the nesting", en los ejemplos de
  rechazo con "<B> is not allowed inside <A>". Sin paso descendiente o sin
  camino, nada (snapshot: solo cambian los casos A//B).
- Plantilla 4.2, S1-00338: //@assyCode[string-length(.) != 2] y objectUse
  "two characters" (solo esa celda).
- Ejemplos editados a mano: siguen sin registrarse, pero el panel lo dice
  junto al veredicto y marca cada ejemplo editado ("Editado"/"Edited");
  Regenerate los quita.
- Tests, caso eval rule-test-4-2-nested-randomlist, simulador y
  verify-rule-test-nesting-and-edits.mjs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rwcp9cSck72V1zULNhL8wU
</commit_message>
<xml_diff>
--- a/public/brdp-template-4-2.xlsx
+++ b/public/brdp-template-4-2.xlsx
@@ -540,8 +540,8 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>&lt;structureObjectRule&gt;
-            &lt;objectPath allowedObjectFlag="0"&gt;//@assyCode[not(matches(., '^\d{2}$'))]&lt;/objectPath&gt;
-            &lt;objectUse&gt;BRDP-S1-00338. The assembly code (@assyCode) must be exactly two digits. &lt;/objectUse&gt;
+            &lt;objectPath allowedObjectFlag="0"&gt;//@assyCode[string-length(.) != 2]&lt;/objectPath&gt;
+            &lt;objectUse&gt;BRDP-S1-00338. The assembly code (@assyCode) must be exactly two characters. &lt;/objectUse&gt;
           &lt;/structureObjectRule&gt;</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Plantillas 4.1/4.2: formato uniforme de las "Note" en Definition
Las Definitions con nota siguen el formato del catálogo 4.2 de sources/:
"Note" en su propia línea, sin líneas en blanco. Cambian solo S1-00150
(4.2, antes "Note:" en línea) y S1-00219 (4.2 y 4.1, antes con líneas en
blanco alrededor). Comprobado celda a celda: ninguna otra celda cambia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rwcp9cSck72V1zULNhL8wU
</commit_message>
<xml_diff>
--- a/public/brdp-template-4-2.xlsx
+++ b/public/brdp-template-4-2.xlsx
@@ -559,7 +559,9 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Decide whether to link from the body of the procedure to the support equipment listed in Preliminary requirements. Note: The attribute id on the element &lt;supportEquipDescr&gt; is used to establish the link between the two and will guarantee consistent use of identification throughout the procedure. The use of cross-references is encouraged.</t>
+          <t>Decide whether to link from the body of the procedure to the support equipment listed in Preliminary requirements.
+Note
+The attribute id on the element &lt;supportEquipDescr&gt; is used to establish the link between the two and will guarantee consistent use of identification throughout the procedure. The use of cross-references is encouraged.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>